<commit_message>
Update Excel Report _7 _Data_Ora_ N_D__Piano_Miglioramento.xlsx
</commit_message>
<xml_diff>
--- a/Piano_Miglioramento/Report _7 _Data_Ora_ N_D__Piano_Miglioramento.xlsx
+++ b/Piano_Miglioramento/Report _7 _Data_Ora_ N_D__Piano_Miglioramento.xlsx
@@ -8,7 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Valutazione del rischio" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Azioni intraprese" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Azioni immediate" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tipologie intervento" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Follow-up azioni" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -450,6 +450,11 @@
           <t>Significatività</t>
         </is>
       </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Sezione Sottosezione</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -472,6 +477,11 @@
       <c r="F2" t="n">
         <v>4</v>
       </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>1. Valutazione del Rischio</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -493,6 +503,11 @@
       </c>
       <c r="F3" t="n">
         <v>9</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>1. Valutazione del Rischio</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -512,19 +527,19 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Tipologia Contenuto</t>
+          <t>Sezione Sottosezione</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Descrizione / Dettaglio</t>
+          <t>Dettaglio / Descrizione</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Azioni immediate di rimedio</t>
+          <t>2. Azioni Immediate di Rimedio</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -544,7 +559,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:C2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -558,6 +573,11 @@
           <t>Descrizione</t>
         </is>
       </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Sezione Sottosezione</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -568,6 +588,11 @@
       <c r="B2" t="inlineStr">
         <is>
           <t>Esempio intervento tecnico correttivo</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>3. Azioni di Miglioramento - Tipologia Intervento</t>
         </is>
       </c>
     </row>
@@ -582,7 +607,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:I2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -626,6 +651,11 @@
           <t>Data e firma</t>
         </is>
       </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Sezione Sottosezione</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -666,6 +696,11 @@
       <c r="H2" t="inlineStr">
         <is>
           <t>2026-06-20 - M. Rossi</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>4. Follow UP Azioni Intraprese</t>
         </is>
       </c>
     </row>

</xml_diff>